<commit_message>
getting it all nice
</commit_message>
<xml_diff>
--- a/output/table3.xlsx
+++ b/output/table3.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="17" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="34" uniqueCount="11">
   <si>
     <t>Panel 1: All Gymnasts</t>
   </si>
@@ -55,7 +55,367 @@
   <numFmts count="1">
     <numFmt numFmtId="166" formatCode="#0.00"/>
   </numFmts>
-  <fonts count="91">
+  <fonts count="181">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -429,7 +789,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="91">
+  <borders count="181">
     <border>
       <left/>
       <right/>
@@ -1067,11 +1427,641 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="181">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -1430,6 +2420,366 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="90" fillId="0" borderId="90" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="91" fillId="0" borderId="91" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="92" fillId="0" borderId="92" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="93" fillId="0" borderId="93" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="94" fillId="0" borderId="94" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="95" fillId="0" borderId="95" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="96" fillId="0" borderId="96" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="97" fillId="0" borderId="97" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="98" fillId="0" borderId="98" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="99" fillId="0" borderId="99" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="100" fillId="0" borderId="100" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="101" fillId="0" borderId="101" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="102" fillId="0" borderId="102" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="103" fillId="0" borderId="103" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="104" fillId="0" borderId="104" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="105" fillId="0" borderId="105" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="106" fillId="0" borderId="106" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="107" fillId="0" borderId="107" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="108" fillId="0" borderId="108" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="109" fillId="0" borderId="109" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="110" fillId="0" borderId="110" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="111" fillId="0" borderId="111" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="112" fillId="0" borderId="112" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="113" fillId="0" borderId="113" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="114" fillId="0" borderId="114" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="115" fillId="0" borderId="115" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="116" fillId="0" borderId="116" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="117" fillId="0" borderId="117" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="118" fillId="0" borderId="118" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="119" fillId="0" borderId="119" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="120" fillId="0" borderId="120" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="121" fillId="0" borderId="121" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="122" fillId="0" borderId="122" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="123" fillId="0" borderId="123" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="124" fillId="0" borderId="124" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="125" fillId="0" borderId="125" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="126" fillId="0" borderId="126" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="127" fillId="0" borderId="127" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="128" fillId="0" borderId="128" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="129" fillId="0" borderId="129" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="130" fillId="0" borderId="130" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="131" fillId="0" borderId="131" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="132" fillId="0" borderId="132" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="133" fillId="0" borderId="133" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="134" fillId="0" borderId="134" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="135" fillId="0" borderId="135" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="136" fillId="0" borderId="136" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="137" fillId="0" borderId="137" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="138" fillId="0" borderId="138" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="139" fillId="0" borderId="139" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="140" fillId="0" borderId="140" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="141" fillId="0" borderId="141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="142" fillId="0" borderId="142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="143" fillId="0" borderId="143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="144" fillId="0" borderId="144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="145" fillId="0" borderId="145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="146" fillId="0" borderId="146" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="147" fillId="0" borderId="147" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="148" fillId="0" borderId="148" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="149" fillId="0" borderId="149" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="150" fillId="0" borderId="150" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="151" fillId="0" borderId="151" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="152" fillId="0" borderId="152" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="153" fillId="0" borderId="153" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="154" fillId="0" borderId="154" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="155" fillId="0" borderId="155" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="156" fillId="0" borderId="156" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="157" fillId="0" borderId="157" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="158" fillId="0" borderId="158" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="159" fillId="0" borderId="159" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="160" fillId="0" borderId="160" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="161" fillId="0" borderId="161" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="162" fillId="0" borderId="162" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="163" fillId="0" borderId="163" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="164" fillId="0" borderId="164" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="165" fillId="0" borderId="165" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="166" fillId="0" borderId="166" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="167" fillId="0" borderId="167" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="168" fillId="0" borderId="168" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="169" fillId="0" borderId="169" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="170" fillId="0" borderId="170" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="171" fillId="0" borderId="171" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="172" fillId="0" borderId="172" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="173" fillId="0" borderId="173" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="174" fillId="0" borderId="174" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="175" fillId="0" borderId="175" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="176" fillId="0" borderId="176" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="177" fillId="0" borderId="177" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="178" fillId="0" borderId="178" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="179" fillId="0" borderId="179" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="180" fillId="0" borderId="180" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1471,36 +2821,36 @@
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="91">
         <v>9.6391804126895</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="92">
         <v>9.5230784480145427</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="93">
         <v>9.5490278913837763</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="94">
         <v>9.6360224743253156</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="95">
         <v>9.586082574146138</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="6">
+      <c r="B4" s="96">
         <v>0.25796401533840307</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="97">
         <v>0.49292093078291382</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="98">
         <v>0.40527700401808497</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="99">
         <v>0.36832135541410371</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="100">
         <v>0.39503591391446152</v>
       </c>
     </row>
@@ -1508,36 +2858,36 @@
       <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="101">
         <v>9.7059091524930619</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="102">
         <v>9.6247883129685139</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="103">
         <v>9.6041886079138195</v>
       </c>
-      <c r="E5" s="14">
+      <c r="E5" s="104">
         <v>9.7213547017138549</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="105">
         <v>9.6721925969287472</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="16">
+      <c r="B6" s="106">
         <v>0.23174365860492571</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="107">
         <v>0.42797971532862361</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="108">
         <v>0.36049745425731022</v>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="109">
         <v>0.33756253849701229</v>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="110">
         <v>0.34124302089971958</v>
       </c>
     </row>
@@ -1545,36 +2895,36 @@
       <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="111">
         <v>9.6557394155248577</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="112">
         <v>9.5474181264606557</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="113">
         <v>9.5720287095896754</v>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="114">
         <v>9.6541143874693134</v>
       </c>
-      <c r="F7" s="25">
+      <c r="F7" s="115">
         <v>9.6072338899952197</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="26">
+      <c r="B8" s="116">
         <v>0.25118517872147778</v>
       </c>
-      <c r="C8" s="27">
+      <c r="C8" s="117">
         <v>0.4784542331536642</v>
       </c>
-      <c r="D8" s="28">
+      <c r="D8" s="118">
         <v>0.39048210145470807</v>
       </c>
-      <c r="E8" s="29">
+      <c r="E8" s="119">
         <v>0.36771558401539112</v>
       </c>
-      <c r="F8" s="30">
+      <c r="F8" s="120">
         <v>0.38385263344989612</v>
       </c>
     </row>
@@ -1587,36 +2937,36 @@
       <c r="A11" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="31">
+      <c r="B11" s="121">
         <v>9.7213286802927801</v>
       </c>
-      <c r="C11" s="32">
+      <c r="C11" s="122">
         <v>9.6619935918992415</v>
       </c>
-      <c r="D11" s="33">
+      <c r="D11" s="123">
         <v>9.6592059847152711</v>
       </c>
-      <c r="E11" s="34">
+      <c r="E11" s="124">
         <v>9.7197856243905871</v>
       </c>
-      <c r="F11" s="35">
+      <c r="F11" s="125">
         <v>9.6901845551774741</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="36">
+      <c r="B12" s="126">
         <v>0.1792917417839377</v>
       </c>
-      <c r="C12" s="37">
+      <c r="C12" s="127">
         <v>0.36205200373424112</v>
       </c>
-      <c r="D12" s="38">
+      <c r="D12" s="128">
         <v>0.30041924047249652</v>
       </c>
-      <c r="E12" s="39">
+      <c r="E12" s="129">
         <v>0.30067857631884359</v>
       </c>
-      <c r="F12" s="40">
+      <c r="F12" s="130">
         <v>0.29575990026060572</v>
       </c>
     </row>
@@ -1624,36 +2974,36 @@
       <c r="A13" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="41">
+      <c r="B13" s="131">
         <v>9.7559224116624677</v>
       </c>
-      <c r="C13" s="42">
+      <c r="C13" s="132">
         <v>9.7041355708345254</v>
       </c>
-      <c r="D13" s="43">
+      <c r="D13" s="133">
         <v>9.6738042952051408</v>
       </c>
-      <c r="E13" s="44">
+      <c r="E13" s="134">
         <v>9.7669488120972758</v>
       </c>
-      <c r="F13" s="45">
+      <c r="F13" s="135">
         <v>9.7315173554660763</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="46">
+      <c r="B14" s="136">
         <v>0.1796300794420275</v>
       </c>
-      <c r="C14" s="47">
+      <c r="C14" s="137">
         <v>0.34618180346929289</v>
       </c>
-      <c r="D14" s="48">
+      <c r="D14" s="138">
         <v>0.29200602477526583</v>
       </c>
-      <c r="E14" s="49">
+      <c r="E14" s="139">
         <v>0.2946794711811257</v>
       </c>
-      <c r="F14" s="50">
+      <c r="F14" s="140">
         <v>0.28048423015781981</v>
       </c>
     </row>
@@ -1661,36 +3011,36 @@
       <c r="A15" t="s">
         <v>3</v>
       </c>
-      <c r="B15" s="51">
+      <c r="B15" s="141">
         <v>9.7281819387260668</v>
       </c>
-      <c r="C15" s="52">
+      <c r="C15" s="142">
         <v>9.6695548550358357</v>
       </c>
-      <c r="D15" s="53">
+      <c r="D15" s="143">
         <v>9.6670916149214126</v>
       </c>
-      <c r="E15" s="54">
+      <c r="E15" s="144">
         <v>9.7287003881941736</v>
       </c>
-      <c r="F15" s="55">
+      <c r="F15" s="145">
         <v>9.6983090516154835</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="56">
+      <c r="B16" s="146">
         <v>0.17999945138972839</v>
       </c>
-      <c r="C16" s="57">
+      <c r="C16" s="147">
         <v>0.36022363050628531</v>
       </c>
-      <c r="D16" s="58">
+      <c r="D16" s="148">
         <v>0.29501979940211198</v>
       </c>
-      <c r="E16" s="59">
+      <c r="E16" s="149">
         <v>0.30877966315912492</v>
       </c>
-      <c r="F16" s="60">
+      <c r="F16" s="150">
         <v>0.29511323759005209</v>
       </c>
     </row>
@@ -1703,36 +3053,36 @@
       <c r="A19" t="s">
         <v>1</v>
       </c>
-      <c r="B19" s="61">
+      <c r="B19" s="151">
         <v>9.398393281224994</v>
       </c>
-      <c r="C19" s="62">
+      <c r="C19" s="152">
         <v>9.1169806207634352</v>
       </c>
-      <c r="D19" s="63">
+      <c r="D19" s="153">
         <v>9.2283144006957318</v>
       </c>
-      <c r="E19" s="64">
+      <c r="E19" s="154">
         <v>9.3867572306159488</v>
       </c>
-      <c r="F19" s="65">
+      <c r="F19" s="155">
         <v>9.2805353092756864</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="66">
+      <c r="B20" s="156">
         <v>0.29937194728338051</v>
       </c>
-      <c r="C20" s="67">
+      <c r="C20" s="157">
         <v>0.5905591830682958</v>
       </c>
-      <c r="D20" s="68">
+      <c r="D20" s="158">
         <v>0.4913981229110338</v>
       </c>
-      <c r="E20" s="69">
+      <c r="E20" s="159">
         <v>0.43281570388803942</v>
       </c>
-      <c r="F20" s="70">
+      <c r="F20" s="160">
         <v>0.48184707759651929</v>
       </c>
     </row>
@@ -1740,36 +3090,36 @@
       <c r="A21" t="s">
         <v>2</v>
       </c>
-      <c r="B21" s="71">
+      <c r="B21" s="161">
         <v>9.4521571780318645</v>
       </c>
-      <c r="C21" s="72">
+      <c r="C21" s="162">
         <v>9.1716974370858892</v>
       </c>
-      <c r="D21" s="73">
+      <c r="D21" s="163">
         <v>9.2891776229205885</v>
       </c>
-      <c r="E21" s="74">
+      <c r="E21" s="164">
         <v>9.4796474626940537</v>
       </c>
-      <c r="F21" s="75">
+      <c r="F21" s="165">
         <v>9.3670254922407565</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="76">
+      <c r="B22" s="166">
         <v>0.29232595807428818</v>
       </c>
-      <c r="C22" s="77">
+      <c r="C22" s="167">
         <v>0.55123899290729783</v>
       </c>
-      <c r="D22" s="78">
+      <c r="D22" s="168">
         <v>0.459610964439714</v>
       </c>
-      <c r="E22" s="79">
+      <c r="E22" s="169">
         <v>0.43406089728606001</v>
       </c>
-      <c r="F22" s="80">
+      <c r="F22" s="170">
         <v>0.44674317027485461</v>
       </c>
     </row>
@@ -1777,36 +3127,36 @@
       <c r="A23" t="s">
         <v>3</v>
       </c>
-      <c r="B23" s="81">
+      <c r="B23" s="171">
         <v>9.4030914534676899</v>
       </c>
-      <c r="C23" s="82">
+      <c r="C23" s="172">
         <v>9.1192248899135002</v>
       </c>
-      <c r="D23" s="83">
+      <c r="D23" s="173">
         <v>9.2402198319010278</v>
       </c>
-      <c r="E23" s="84">
+      <c r="E23" s="174">
         <v>9.3937756171708457</v>
       </c>
-      <c r="F23" s="85">
+      <c r="F23" s="175">
         <v>9.2890571195611855</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="86">
+      <c r="B24" s="176">
         <v>0.29667071966902192</v>
       </c>
-      <c r="C24" s="87">
+      <c r="C24" s="177">
         <v>0.58388619082825155</v>
       </c>
-      <c r="D24" s="88">
+      <c r="D24" s="178">
         <v>0.48914491820846451</v>
       </c>
-      <c r="E24" s="89">
+      <c r="E24" s="179">
         <v>0.43266328578446228</v>
       </c>
-      <c r="F24" s="90">
+      <c r="F24" s="180">
         <v>0.47709825129063271</v>
       </c>
     </row>

</xml_diff>